<commit_message>
chore: added add app launcher on the excel file
</commit_message>
<xml_diff>
--- a/DOCUMENTATION/zyphor-project-inventory.xlsx
+++ b/DOCUMENTATION/zyphor-project-inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\kali-linux\home\programmer\zyphor-os-desktop\DOCUMENTATION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC22C948-F913-49DD-990F-C785B8423125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{759FCC5B-ABEF-4510-AD9D-1168C1EB1EAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32205" yWindow="2370" windowWidth="21600" windowHeight="12720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29580" yWindow="780" windowWidth="21600" windowHeight="12720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="122">
   <si>
     <t>Packages</t>
   </si>
@@ -388,6 +388,9 @@
   </si>
   <si>
     <t>rm jul 24, 2027</t>
+  </si>
+  <si>
+    <t>add app launcher</t>
   </si>
 </sst>
 </file>
@@ -480,9 +483,6 @@
   </cellStyleXfs>
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -491,6 +491,9 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -768,22 +771,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="I1" s="1" t="s">
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="I1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="1"/>
-      <c r="L1" s="2" t="s">
+      <c r="J1" s="9"/>
+      <c r="L1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="N1" s="2"/>
+      <c r="N1" s="1"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
@@ -818,27 +821,27 @@
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3" t="s">
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" s="3"/>
-      <c r="I3" s="4" t="s">
+      <c r="F3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="I3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="J3" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L3" t="s">
@@ -846,27 +849,27 @@
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3" t="s">
+      <c r="D4" s="2"/>
+      <c r="E4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G4" s="3"/>
-      <c r="I4" s="4" t="s">
+      <c r="F4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="I4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="J4" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L4" t="s">
@@ -874,27 +877,27 @@
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3" t="s">
+      <c r="D5" s="2"/>
+      <c r="E5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G5" s="3"/>
-      <c r="I5" s="4" t="s">
+      <c r="F5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="2"/>
+      <c r="I5" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="J5" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L5" t="s">
@@ -902,10 +905,10 @@
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="I6" s="4" t="s">
+      <c r="I6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="J6" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L6" t="s">
@@ -913,27 +916,27 @@
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4" t="s">
+      <c r="D7" s="3"/>
+      <c r="E7" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G7" s="4"/>
-      <c r="I7" s="4" t="s">
+      <c r="F7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="3"/>
+      <c r="I7" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="J7" s="4" t="s">
+      <c r="J7" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L7" t="s">
@@ -941,27 +944,27 @@
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4" t="s">
+      <c r="D8" s="3"/>
+      <c r="E8" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F8" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G8" s="4"/>
-      <c r="I8" s="4" t="s">
+      <c r="F8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="3"/>
+      <c r="I8" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="J8" s="4" t="s">
+      <c r="J8" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L8" t="s">
@@ -969,535 +972,538 @@
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4" t="s">
+      <c r="D9" s="3"/>
+      <c r="E9" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="F9" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G9" s="4"/>
-      <c r="I9" s="5" t="s">
+      <c r="F9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G9" s="3"/>
+      <c r="I9" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="J9" s="5" t="s">
-        <v>44</v>
+      <c r="J9" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="L9" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4" t="s">
+      <c r="D10" s="3"/>
+      <c r="E10" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F10" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G10" s="4"/>
-      <c r="I10" s="5" t="s">
+      <c r="F10" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G10" s="3"/>
+      <c r="I10" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="J10" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="L10" t="s">
+      <c r="J10" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G11" s="3"/>
+      <c r="I11" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="L11" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C11" s="4" t="s">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4" t="s">
+      <c r="D12" s="3"/>
+      <c r="E12" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G12" s="3"/>
+      <c r="I12" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="L12" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G13" s="3"/>
+      <c r="I13" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="L13" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="L14" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I15" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="L15" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G11" s="4"/>
-      <c r="I11" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="J11" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="L11" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+      <c r="F16" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" s="5"/>
+      <c r="I16" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="L16" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G17" s="5"/>
+      <c r="I17" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="L17" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G18" s="5"/>
+      <c r="I18" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I19" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="J19" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G20" s="5"/>
+      <c r="I20" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G21" s="5"/>
+      <c r="I21" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G22" s="5"/>
+      <c r="I22" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J22" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I23" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="J23" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I24" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="J24" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I25" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="J25" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I26" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J26" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I27" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J27" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I28" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="J28" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I29" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G12" s="4"/>
-      <c r="I12" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="J12" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="L12" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G13" s="4"/>
-      <c r="I13" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="J13" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="L13" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="I14" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="J14" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="L14" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="I15" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="J15" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="L15" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="G16" s="6"/>
-      <c r="I16" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="J16" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="L16" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="G17" s="6"/>
-      <c r="I17" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="J17" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="G18" s="6"/>
-      <c r="I18" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="J18" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I19" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="J19" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="G20" s="6"/>
-      <c r="I20" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="J20" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A21" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="G21" s="6"/>
-      <c r="I21" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="J21" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="G22" s="6"/>
-      <c r="I22" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="J22" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I23" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="J23" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I24" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="J24" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I25" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="J25" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I26" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="J26" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I27" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="J27" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I28" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="J28" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I29" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="J29" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I30" s="5" t="s">
+      <c r="J29" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I30" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="J30" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I31" s="5" t="s">
+      <c r="J30" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I31" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="J31" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I32" s="5" t="s">
+      <c r="J31" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I32" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="J32" s="5" t="s">
+      <c r="J32" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="33" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="I33" s="5" t="s">
+      <c r="I33" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="J33" s="5" t="s">
+      <c r="J33" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="34" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="I34" s="5" t="s">
+      <c r="I34" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="J34" s="5" t="s">
+      <c r="J34" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="35" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="I35" s="5" t="s">
+      <c r="I35" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="J35" s="5" t="s">
+      <c r="J35" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="36" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="I36" s="5" t="s">
+      <c r="I36" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="J36" s="5" t="s">
+      <c r="J36" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="37" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="I37" s="5" t="s">
+      <c r="I37" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="J37" s="5" t="s">
+      <c r="J37" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="38" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="I38" s="5" t="s">
+      <c r="I38" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="J38" s="5" t="s">
+      <c r="J38" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="39" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="I39" s="5" t="s">
+      <c r="I39" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="J39" s="5" t="s">
+      <c r="J39" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="40" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="I40" s="5" t="s">
+      <c r="I40" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="J40" s="5" t="s">
+      <c r="J40" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="41" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="I41" s="5" t="s">
+      <c r="I41" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="J41" s="5" t="s">
+      <c r="J41" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="42" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="I42" s="5" t="s">
+      <c r="I42" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="J42" s="5" t="s">
+      <c r="J42" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="43" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="I43" s="5" t="s">
+      <c r="I43" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="J43" s="5" t="s">
+      <c r="J43" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="44" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="I44" s="5" t="s">
+      <c r="I44" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="J44" s="5" t="s">
+      <c r="J44" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="45" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="I45" s="5" t="s">
+      <c r="I45" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="J45" s="5" t="s">
+      <c r="J45" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="46" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="I46" s="5" t="s">
+      <c r="I46" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="J46" s="5" t="s">
+      <c r="J46" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="47" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="I47" s="7" t="s">
+      <c r="I47" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="J47" s="7" t="s">
+      <c r="J47" s="6" t="s">
         <v>44</v>
       </c>
       <c r="K47" t="s">
@@ -1505,66 +1511,66 @@
       </c>
     </row>
     <row r="48" spans="9:11" x14ac:dyDescent="0.25">
-      <c r="I48" s="5" t="s">
+      <c r="I48" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="J48" s="5" t="s">
+      <c r="J48" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="49" spans="9:10" x14ac:dyDescent="0.25">
-      <c r="I49" s="5" t="s">
+      <c r="I49" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="J49" s="5" t="s">
+      <c r="J49" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="50" spans="9:10" x14ac:dyDescent="0.25">
-      <c r="I50" s="5" t="s">
+      <c r="I50" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="J50" s="5" t="s">
+      <c r="J50" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="51" spans="9:10" x14ac:dyDescent="0.25">
-      <c r="I51" s="9" t="s">
+      <c r="I51" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="J51" s="9" t="s">
+      <c r="J51" s="8" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="52" spans="9:10" x14ac:dyDescent="0.25">
-      <c r="I52" s="8" t="s">
+      <c r="I52" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="J52" s="8" t="s">
+      <c r="J52" s="7" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="53" spans="9:10" x14ac:dyDescent="0.25">
-      <c r="I53" s="3" t="s">
+      <c r="I53" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="J53" s="3" t="s">
+      <c r="J53" s="2" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="54" spans="9:10" x14ac:dyDescent="0.25">
-      <c r="I54" s="3" t="s">
+      <c r="I54" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="J54" s="3" t="s">
+      <c r="J54" s="2" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="55" spans="9:10" x14ac:dyDescent="0.25">
-      <c r="I55" s="3" t="s">
+      <c r="I55" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="J55" s="3" t="s">
+      <c r="J55" s="2" t="s">
         <v>86</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: modified excel file
</commit_message>
<xml_diff>
--- a/DOCUMENTATION/zyphor-project-inventory.xlsx
+++ b/DOCUMENTATION/zyphor-project-inventory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\kali-linux\home\programmer\zyphor-os-desktop\DOCUMENTATION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{759FCC5B-ABEF-4510-AD9D-1168C1EB1EAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55066A53-1F9A-4536-ACC2-BA718810949F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29580" yWindow="780" windowWidth="21600" windowHeight="12720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29925" yWindow="1125" windowWidth="21600" windowHeight="12720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>